<commit_message>
Ny kode for NR med pandapower
</commit_message>
<xml_diff>
--- a/Grid/test_trøndelagsnettet_ny.xlsx
+++ b/Grid/test_trøndelagsnettet_ny.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b57458e082dedb4f/Dokumenter/EMIL 1. klasse høst/TET4205 Power system analysis 2/Kraftsystemer-2/Grid/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="8_{656A97CD-AEDD-46F6-9589-F7560D954F76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A25991C8-C88D-4457-8DF1-5719B1C3496B}"/>
+  <xr:revisionPtr revIDLastSave="22" documentId="8_{656A97CD-AEDD-46F6-9589-F7560D954F76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{84E69CE6-C95C-447E-B40E-C5FEDB1C1AA6}"/>
   <bookViews>
-    <workbookView xWindow="-86" yWindow="0" windowWidth="12515" windowHeight="14794" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14914" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="bus" sheetId="1" r:id="rId1"/>
@@ -789,10 +789,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5038,7 +5034,7 @@
   <cols>
     <col min="9" max="9" width="11.3046875" customWidth="1"/>
     <col min="10" max="10" width="13.23046875" customWidth="1"/>
-    <col min="12" max="12" width="0" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="12.53515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">

</xml_diff>

<commit_message>
Oppdatert pandapower og Newton-Raphson
</commit_message>
<xml_diff>
--- a/Grid/test_trøndelagsnettet_ny.xlsx
+++ b/Grid/test_trøndelagsnettet_ny.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="22" documentId="8_{656A97CD-AEDD-46F6-9589-F7560D954F76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{84E69CE6-C95C-447E-B40E-C5FEDB1C1AA6}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14914" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14914" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="bus" sheetId="1" r:id="rId1"/>
@@ -789,6 +789,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>